<commit_message>
Update reports 2026-09-01 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-01.xlsx
+++ b/gex_pivot_levels_2026-09-01.xlsx
@@ -15,12 +15,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Pivots" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ES'!$A$1:$G$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'NQ'!$A$1:$G$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RTY'!$A$1:$G$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'CL'!$A$1:$G$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'GC'!$A$1:$G$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'All Pivots'!$A$1:$H$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -544,12 +544,12 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>-$5.49M</t>
+          <t>-$6.15M</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>+$9.58M</t>
+          <t>+$10.74M</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>-$6.38M</t>
+          <t>-$7.15M</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>+$8.16M</t>
+          <t>+$9.14M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -639,12 +639,12 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>-$2.46M</t>
+          <t>-$2.72M</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>+$7.94M</t>
+          <t>+$8.78M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>-$8.18M</t>
+          <t>-$8.95M</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>+$19.28M</t>
+          <t>+$21.09M</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -721,33 +721,33 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="6" t="n">
         <v>7672.86</v>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="6" t="n">
         <v>7660</v>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>-$9.47M</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>+$12.20M</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>-$10.19M</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>+$13.14M</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -800,12 +800,12 @@
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>+$197.07K</t>
+          <t>+$407.67K</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>+$37.56M</t>
+          <t>+$39.29M</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -866,12 +866,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>-$7.24M</t>
+          <t>-$7.38M</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$22.98M</t>
+          <t>+$23.43M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -887,10 +887,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>7697.86</v>
+        <v>7702.86</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>7685</v>
+        <v>7690</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
@@ -899,64 +899,56 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>-$2.78M</t>
+          <t>-$6.03M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$18.99M</t>
+          <t>+$30.51M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n">
-        <v>7702.86</v>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>7690</v>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="A14" s="2" t="n">
+        <v>7712.86</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>7700</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>-$6.26M</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>+$30.98M</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G14" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>+$5.02M</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>+$31.18M</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>7712.86</v>
+        <v>7717.86</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>7700</v>
+        <v>7705</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
@@ -965,41 +957,45 @@
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>+$5.28M</t>
+          <t>+$12.11M</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$32.77M</t>
+          <t>+$17.18M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>7717.86</v>
+        <v>7718.54</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>7705</v>
+        <v>769</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>+$12.90M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>-$4.40M</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>+$18.30M</t>
+          <t>+$19.01M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -1009,158 +1005,158 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>7718.54</v>
+        <v>7727.86</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>769</v>
+        <v>7715</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>+$5.56M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>+$13.82M</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>7728.56</v>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>770</v>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>-$4.40M</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>+$19.01M</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
-        <v>7727.86</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>7715</v>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>+$7.58M</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>+$39.37M</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>7737.86</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>7725</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>+$6.16M</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>+$15.29M</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="n">
-        <v>7728.56</v>
-      </c>
-      <c r="B19" s="6" t="n">
-        <v>770</v>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>+$7.58M</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>+$39.37M</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>+$6.76M</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>+$19.26M</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>7737.86</v>
+        <v>7738.58</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7725</v>
+        <v>771</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>+$7.72M</t>
+          <t>+$1.99M</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+$22.01M</t>
+          <t>+$17.54M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>7738.58</v>
+        <v>7742.86</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>771</v>
+        <v>7730</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>+$1.99M</t>
+          <t>+$9.25M</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>+$17.54M</t>
+          <t>+$12.71M</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -1170,16 +1166,16 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>7742.86</v>
+        <v>7747.86</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>7730</v>
+        <v>7735</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
@@ -1188,12 +1184,12 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>+$10.60M</t>
+          <t>+$4.23M</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>+$14.56M</t>
+          <t>+$6.20M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1203,206 +1199,173 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>7747.86</v>
+        <v>7748.6</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>7735</v>
+        <v>772</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>+$10.64M</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>+$18.48M</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>7752.86</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>7740</v>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>+$4.99M</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>+$7.31M</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>7748.6</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>772</v>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>+$10.64M</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>+$18.48M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>+$7.73M</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>+$11.36M</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n">
-        <v>7752.86</v>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>7740</v>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="A25" s="2" t="n">
+        <v>7762.86</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>7750</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>+$9.18M</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>+$13.49M</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>+$6.29M</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>+$9.10M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>7762.86</v>
+        <v>7768.64</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>7750</v>
+        <v>774</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>SPY</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>+$7.15M</t>
+          <t>+$1.95M</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>+$10.34M</t>
+          <t>+$5.65M</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>7768.64</v>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>774</v>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="A27" s="6" t="n">
+        <v>7778.66</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>775</v>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>+$1.95M</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr">
-        <is>
-          <t>+$5.65M</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="n">
-        <v>7778.66</v>
-      </c>
-      <c r="B28" s="6" t="n">
-        <v>775</v>
-      </c>
-      <c r="C28" s="7" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>+$7.38M</t>
         </is>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>+$9.04M</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G28"/>
+  <autoFilter ref="A1:G27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3351,7 +3314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3463,12 +3426,12 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>+$197.07K</t>
+          <t>+$407.67K</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>+$37.56M</t>
+          <t>+$39.29M</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -3501,12 +3464,12 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>+$5.28M</t>
+          <t>+$5.02M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$32.77M</t>
+          <t>+$31.18M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3517,42 +3480,38 @@
       <c r="H4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="2" t="n">
         <v>7702.86</v>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="2" t="n">
         <v>7690</v>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>-$6.26M</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>+$30.98M</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>-$6.03M</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>+$30.51M</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -3611,12 +3570,12 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>-$7.24M</t>
+          <t>-$7.38M</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>+$22.98M</t>
+          <t>+$23.43M</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -3637,24 +3596,24 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>7737.86</v>
+        <v>7662.86</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7725</v>
+        <v>7650</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>+$7.72M</t>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>-$8.95M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>+$22.01M</t>
+          <t>+$21.09M</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3747,24 +3706,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>7662.86</v>
+        <v>7737.86</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>7650</v>
+        <v>7725</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>-$8.18M</t>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>+$6.76M</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>+$19.28M</t>
+          <t>+$19.26M</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
@@ -3819,24 +3778,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>7697.86</v>
+        <v>7748.6</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>7685</v>
+        <v>772</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>-$2.78M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>+$10.64M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>+$18.99M</t>
+          <t>+$18.48M</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -3857,10 +3816,10 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>7748.6</v>
+        <v>7738.58</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
@@ -3869,12 +3828,12 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>+$10.64M</t>
+          <t>+$1.99M</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>+$18.48M</t>
+          <t>+$17.54M</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -3884,7 +3843,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3907,12 +3866,12 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>+$12.90M</t>
+          <t>+$12.11M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>+$18.30M</t>
+          <t>+$17.18M</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
@@ -3929,74 +3888,74 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>7738.58</v>
+        <v>29522.86</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>771</v>
+        <v>717</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>+$1.99M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>-$1.25M</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>+$17.54M</t>
+          <t>+$16.50M</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
-        <v>29522.86</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>717</v>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="B17" s="6" t="n">
+        <v>29646.16</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>720</v>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>-$1.25M</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>+$16.50M</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr"/>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>+$5.50M</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>+$15.86M</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -4005,10 +3964,10 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>29646.16</v>
+        <v>29851.64</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
@@ -4017,12 +3976,12 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>+$5.50M</t>
+          <t>+$11.59M</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>+$15.86M</t>
+          <t>+$14.35M</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -4055,12 +4014,12 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>+$6.16M</t>
+          <t>+$5.56M</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>+$15.29M</t>
+          <t>+$13.82M</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
@@ -4077,66 +4036,62 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7742.86</v>
+        <v>29235.18</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>7730</v>
+        <v>710</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>+$10.60M</t>
+          <t>+$1.25M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>+$14.56M</t>
+          <t>+$13.54M</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>29851.64</v>
+        <v>7672.86</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>725</v>
+        <v>7660</v>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>+$11.59M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>-$10.19M</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>+$14.35M</t>
+          <t>+$13.14M</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -4146,293 +4101,297 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>29235.18</v>
+        <v>7742.86</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>710</v>
+        <v>7730</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
+          <t>SPX</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>+$1.25M</t>
+          <t>+$9.25M</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>+$13.54M</t>
+          <t>+$12.71M</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>4636.75</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>102</v>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>+$10.79M</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>+$11.75M</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n">
+      <c r="B24" s="6" t="n">
         <v>7752.86</v>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C24" s="6" t="n">
         <v>7740</v>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>+$9.18M</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>+$13.49M</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>+$7.73M</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>+$11.36M</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>7672.86</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>7660</v>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>-$9.47M</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>+$12.20M</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>29563.96</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>718</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>-$2.33M</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>+$10.94M</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>4636.75</v>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>102</v>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>+$10.79M</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>+$11.75M</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>7637.86</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>7625</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>-$6.15M</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>+$10.74M</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
-        <v>29563.96</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>718</v>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="B27" s="6" t="n">
+        <v>29728.35</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>722</v>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>-$2.33M</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>+$10.94M</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>+$1.53M</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>+$10.25M</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
-        <v>7762.86</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>7750</v>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>+$7.15M</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>+$10.34M</t>
-        </is>
-      </c>
-      <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="n">
-        <v>29728.35</v>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>722</v>
-      </c>
-      <c r="D28" s="7" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>+$1.53M</t>
-        </is>
-      </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>+$10.25M</t>
-        </is>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H28" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="B28" s="2" t="n">
+        <v>7668.44</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>764</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>+$744.47K</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>+$10.03M</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>7668.44</v>
+        <v>29481.77</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>764</v>
+        <v>716</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>SPY</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>+$744.47K</t>
+          <t>+$1.64M</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>+$10.03M</t>
+          <t>+$9.99M</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
@@ -4449,28 +4408,28 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
-        <v>29481.77</v>
+        <v>7652.86</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>716</v>
+        <v>7640</v>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>+$1.64M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>-$7.15M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$9.99M</t>
+          <t>+$9.14M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -4480,7 +4439,7 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -4491,24 +4450,24 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>7637.86</v>
+        <v>7762.86</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>7625</v>
+        <v>7750</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>-$5.49M</t>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>+$6.29M</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>+$9.58M</t>
+          <t>+$9.10M</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -4557,144 +4516,144 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>7657.86</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>7645</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>-$2.72M</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>+$8.78M</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>RTY</t>
         </is>
       </c>
-      <c r="B33" s="6" t="n">
+      <c r="B34" s="6" t="n">
         <v>2947.58</v>
       </c>
-      <c r="C33" s="6" t="n">
+      <c r="C34" s="6" t="n">
         <v>293</v>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>IWM</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>-$6.67M</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>+$8.35M</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G34" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
+      <c r="H34" s="7" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="n">
-        <v>7652.86</v>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>7640</v>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>-$6.38M</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>+$8.16M</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>4364</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>-$7.54M</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>+$7.90M</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>7657.86</v>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>7645</v>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>-$2.46M</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>+$7.94M</t>
-        </is>
-      </c>
-      <c r="G35" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B36" s="6" t="n">
-        <v>4364</v>
+        <v>2977.76</v>
       </c>
       <c r="C36" s="6" t="n">
-        <v>96</v>
+        <v>296</v>
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>GDX</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>-$7.54M</t>
+          <t>-$3.97M</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>+$7.90M</t>
+          <t>+$7.15M</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -4711,74 +4670,74 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>4545.83</v>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>-$4.65M</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>+$6.48M</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
-        <v>7747.86</v>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>7735</v>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>+$4.99M</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>+$7.31M</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="n">
-        <v>2977.76</v>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>296</v>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>-$3.97M</t>
-        </is>
-      </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>+$7.15M</t>
-        </is>
-      </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H38" s="7" t="inlineStr">
+      <c r="B38" s="2" t="n">
+        <v>7638.38</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>761</v>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>-$4.92M</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>+$6.42M</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>valley</t>
         </is>
@@ -4787,188 +4746,188 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>7747.86</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>7735</v>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>+$4.23M</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>+$6.20M</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>29317.38</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>712</v>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>-$3.10M</t>
+        </is>
+      </c>
+      <c r="F40" s="7" t="inlineStr">
+        <is>
+          <t>+$5.72M</t>
+        </is>
+      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>7768.64</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>774</v>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>+$1.95M</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>+$5.65M</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
-        <v>4545.83</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="B42" s="6" t="n">
+        <v>4818.58</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>106</v>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
         <is>
           <t>GDX</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>-$4.65M</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>+$6.48M</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>7638.38</v>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>761</v>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>-$4.92M</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>+$6.42M</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="n">
-        <v>29317.38</v>
-      </c>
-      <c r="C41" s="6" t="n">
-        <v>712</v>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>-$3.10M</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>+$5.72M</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>+$5.33M</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>+$5.36M</t>
+        </is>
+      </c>
+      <c r="G42" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H41" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="n">
-        <v>7768.64</v>
-      </c>
-      <c r="C42" s="2" t="n">
-        <v>774</v>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>+$1.95M</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>+$5.65M</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="H42" s="7" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n">
-        <v>4818.58</v>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>106</v>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E43" s="9" t="inlineStr">
-        <is>
-          <t>+$5.33M</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>+$5.36M</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H43" s="7" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>2967.7</v>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>295</v>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>-$1.14M</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>+$4.80M</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -4977,28 +4936,28 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
-        <v>2967.7</v>
+        <v>29358.47</v>
       </c>
       <c r="C44" s="2" t="n">
-        <v>295</v>
+        <v>713</v>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>-$1.14M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>+$210.33K</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>+$4.80M</t>
+          <t>+$4.05M</t>
         </is>
       </c>
       <c r="G44" s="3" t="inlineStr">
@@ -5013,68 +4972,68 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="n">
-        <v>29358.47</v>
-      </c>
-      <c r="C45" s="2" t="n">
-        <v>713</v>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>+$210.33K</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr">
-        <is>
-          <t>+$4.05M</t>
-        </is>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>4484.46</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>409</v>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>-$3.47M</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>+$3.69M</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>RTY</t>
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>4484.46</v>
+        <v>2917.4</v>
       </c>
       <c r="C46" s="6" t="n">
-        <v>409</v>
+        <v>290</v>
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>GLD</t>
+          <t>IWM</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>-$3.47M</t>
+          <t>-$3.57M</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>+$3.69M</t>
+          <t>+$3.57M</t>
         </is>
       </c>
       <c r="G46" s="7" t="inlineStr">
@@ -5091,28 +5050,28 @@
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>RTY</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B47" s="6" t="n">
-        <v>2917.4</v>
+        <v>84.73999999999999</v>
       </c>
       <c r="C47" s="6" t="n">
-        <v>290</v>
+        <v>132</v>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E47" s="8" t="inlineStr">
-        <is>
-          <t>-$3.57M</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>+$1.76M</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>+$3.57M</t>
+          <t>+$2.15M</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -5122,81 +5081,81 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>4409.46</v>
+      </c>
+      <c r="C48" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>-$1.69M</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>+$1.81M</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B48" s="6" t="n">
-        <v>84.73999999999999</v>
-      </c>
-      <c r="C48" s="6" t="n">
-        <v>132</v>
-      </c>
-      <c r="D48" s="7" t="inlineStr">
+      <c r="B49" s="6" t="n">
+        <v>83.45</v>
+      </c>
+      <c r="C49" s="6" t="n">
+        <v>130</v>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr">
-        <is>
-          <t>+$1.76M</t>
-        </is>
-      </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>+$2.15M</t>
-        </is>
-      </c>
-      <c r="G48" s="7" t="inlineStr">
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>+$1.36M</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>+$1.80M</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="n">
-        <v>4409.46</v>
-      </c>
-      <c r="C49" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>-$1.69M</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr">
-        <is>
-          <t>+$1.81M</t>
-        </is>
-      </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr">
+      <c r="H49" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5209,10 +5168,10 @@
         </is>
       </c>
       <c r="B50" s="6" t="n">
-        <v>83.45</v>
+        <v>89.87</v>
       </c>
       <c r="C50" s="6" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
@@ -5221,12 +5180,12 @@
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>+$1.36M</t>
+          <t>+$1.65M</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>+$1.80M</t>
+          <t>+$1.79M</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -5241,76 +5200,76 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="7" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>RTY</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="n">
+        <v>2937.52</v>
+      </c>
+      <c r="C51" s="2" t="n">
+        <v>292</v>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>IWM</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>-$1.62M</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>+$1.74M</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="B51" s="6" t="n">
-        <v>89.87</v>
-      </c>
-      <c r="C51" s="6" t="n">
-        <v>140</v>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="B52" s="6" t="n">
+        <v>86.66</v>
+      </c>
+      <c r="C52" s="6" t="n">
+        <v>135</v>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>USO</t>
         </is>
       </c>
-      <c r="E51" s="9" t="inlineStr">
-        <is>
-          <t>+$1.65M</t>
-        </is>
-      </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>+$1.79M</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>+$1.24M</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>+$1.37M</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>RTY</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="n">
-        <v>2937.52</v>
-      </c>
-      <c r="C52" s="2" t="n">
-        <v>292</v>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>IWM</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>-$1.62M</t>
-        </is>
-      </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>+$1.74M</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
@@ -5319,28 +5278,28 @@
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>GC</t>
         </is>
       </c>
       <c r="B53" s="6" t="n">
-        <v>86.66</v>
+        <v>4440.6</v>
       </c>
       <c r="C53" s="6" t="n">
-        <v>135</v>
+        <v>405</v>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E53" s="9" t="inlineStr">
-        <is>
-          <t>+$1.24M</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>-$742.12K</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>+$1.37M</t>
+          <t>+$1.32M</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -5350,119 +5309,115 @@
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="n">
+        <v>4517.35</v>
+      </c>
+      <c r="C54" s="2" t="n">
+        <v>412</v>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>+$239.16K</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>+$813.71K</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>NQ</t>
+        </is>
+      </c>
+      <c r="B55" s="6" t="n">
+        <v>29496.03</v>
+      </c>
+      <c r="C55" s="6" t="n">
+        <v>29440</v>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E55" s="9" t="inlineStr">
+        <is>
+          <t>+$630.97K</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>+$741.14K</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>GC</t>
         </is>
       </c>
-      <c r="B54" s="6" t="n">
-        <v>4440.6</v>
-      </c>
-      <c r="C54" s="6" t="n">
-        <v>405</v>
-      </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="B56" s="2" t="n">
+        <v>4539.28</v>
+      </c>
+      <c r="C56" s="2" t="n">
+        <v>414</v>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>GLD</t>
         </is>
       </c>
-      <c r="E54" s="8" t="inlineStr">
-        <is>
-          <t>-$742.12K</t>
-        </is>
-      </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>+$1.32M</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H54" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="n">
-        <v>4517.35</v>
-      </c>
-      <c r="C55" s="2" t="n">
-        <v>412</v>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
-        <is>
-          <t>+$239.16K</t>
-        </is>
-      </c>
-      <c r="F55" s="3" t="inlineStr">
-        <is>
-          <t>+$813.71K</t>
-        </is>
-      </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>-$15.97K</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>+$621.74K</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H55" s="3" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B56" s="6" t="n">
-        <v>29496.03</v>
-      </c>
-      <c r="C56" s="6" t="n">
-        <v>29440</v>
-      </c>
-      <c r="D56" s="7" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E56" s="9" t="inlineStr">
-        <is>
-          <t>+$630.97K</t>
-        </is>
-      </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>+$741.14K</t>
-        </is>
-      </c>
-      <c r="G56" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H56" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="H56" s="3" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -5471,32 +5426,36 @@
         </is>
       </c>
       <c r="B57" s="2" t="n">
-        <v>4539.28</v>
+        <v>4682.21</v>
       </c>
       <c r="C57" s="2" t="n">
-        <v>414</v>
+        <v>103</v>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E57" s="4" t="inlineStr">
-        <is>
-          <t>-$15.97K</t>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>+$159.12K</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>+$621.74K</t>
+          <t>+$596.26K</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
@@ -5505,62 +5464,58 @@
         </is>
       </c>
       <c r="B58" s="2" t="n">
-        <v>4682.21</v>
+        <v>4385.78</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>103</v>
+        <v>400</v>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E58" s="5" t="inlineStr">
-        <is>
-          <t>+$159.12K</t>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>-$543.71K</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>+$596.26K</t>
+          <t>+$557.63K</t>
         </is>
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>4385.78</v>
+        <v>29556.03</v>
       </c>
       <c r="C59" s="2" t="n">
-        <v>400</v>
+        <v>29500</v>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>-$543.71K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>+$111.35K</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>+$557.63K</t>
+          <t>+$524.92K</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -5573,62 +5528,66 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>29556.03</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="C60" s="2" t="n">
-        <v>29500</v>
+        <v>131</v>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>+$111.35K</t>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>-$92.83K</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>+$524.92K</t>
+          <t>+$498.84K</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>84.09999999999999</v>
+        <v>29506.03</v>
       </c>
       <c r="C61" s="2" t="n">
-        <v>131</v>
+        <v>29450</v>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E61" s="4" t="inlineStr">
-        <is>
-          <t>-$92.83K</t>
+          <t>NDX</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>+$75.12K</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>+$498.84K</t>
+          <t>+$455.70K</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -5645,28 +5604,28 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>29506.03</v>
+        <v>85.38</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>29450</v>
+        <v>133</v>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>+$75.12K</t>
+          <t>+$156.10K</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>+$455.70K</t>
+          <t>+$414.56K</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -5687,10 +5646,10 @@
         </is>
       </c>
       <c r="B63" s="2" t="n">
-        <v>85.38</v>
+        <v>88.59</v>
       </c>
       <c r="C63" s="2" t="n">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
@@ -5699,58 +5658,58 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>+$156.10K</t>
+          <t>+$247.08K</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>+$414.56K</t>
+          <t>+$341.10K</t>
         </is>
       </c>
       <c r="G63" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>88.59</v>
+        <v>29526.03</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>138</v>
+        <v>29470</v>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>+$247.08K</t>
+          <t>+$291.62K</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>+$341.10K</t>
+          <t>+$312.83K</t>
         </is>
       </c>
       <c r="G64" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
@@ -5759,10 +5718,10 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>29526.03</v>
+        <v>29616.03</v>
       </c>
       <c r="C65" s="2" t="n">
-        <v>29470</v>
+        <v>29560</v>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
@@ -5771,122 +5730,118 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>+$291.62K</t>
+          <t>+$130.20K</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>+$312.83K</t>
+          <t>+$260.40K</t>
         </is>
       </c>
       <c r="G65" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B66" s="2" t="n">
-        <v>29616.03</v>
-      </c>
-      <c r="C66" s="2" t="n">
-        <v>29560</v>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="B66" s="6" t="n">
+        <v>29536.03</v>
+      </c>
+      <c r="C66" s="6" t="n">
+        <v>29480</v>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E66" s="5" t="inlineStr">
-        <is>
-          <t>+$130.20K</t>
-        </is>
-      </c>
-      <c r="F66" s="3" t="inlineStr">
-        <is>
-          <t>+$260.40K</t>
-        </is>
-      </c>
-      <c r="G66" s="3" t="inlineStr">
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>-$132.56K</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>+$249.21K</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="n">
+        <v>77.04000000000001</v>
+      </c>
+      <c r="C67" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>USO</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>-$235.22K</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>+$247.83K</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
         <is>
           <t>Abs</t>
         </is>
       </c>
-      <c r="H66" s="3" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="7" t="inlineStr">
-        <is>
-          <t>NQ</t>
-        </is>
-      </c>
-      <c r="B67" s="6" t="n">
-        <v>29536.03</v>
-      </c>
-      <c r="C67" s="6" t="n">
-        <v>29480</v>
-      </c>
-      <c r="D67" s="7" t="inlineStr">
-        <is>
-          <t>NDX</t>
-        </is>
-      </c>
-      <c r="E67" s="8" t="inlineStr">
-        <is>
-          <t>-$132.56K</t>
-        </is>
-      </c>
-      <c r="F67" s="7" t="inlineStr">
-        <is>
-          <t>+$249.21K</t>
-        </is>
-      </c>
-      <c r="G67" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H67" s="7" t="inlineStr">
-        <is>
-          <t>valley</t>
-        </is>
-      </c>
+      <c r="H67" s="3" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>CL</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>77.04000000000001</v>
+        <v>29456.03</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>120</v>
+        <v>29400</v>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>USO</t>
+          <t>NDX</t>
         </is>
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
-          <t>-$235.22K</t>
+          <t>-$61.27K</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>+$247.83K</t>
+          <t>+$230.94K</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -5903,10 +5858,10 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>29456.03</v>
+        <v>29706.03</v>
       </c>
       <c r="C69" s="2" t="n">
-        <v>29400</v>
+        <v>29650</v>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
@@ -5915,12 +5870,12 @@
       </c>
       <c r="E69" s="4" t="inlineStr">
         <is>
-          <t>-$61.27K</t>
+          <t>-$49.78K</t>
         </is>
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>+$230.94K</t>
+          <t>+$218.28K</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -5937,146 +5892,146 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>29706.03</v>
+        <v>29576.03</v>
       </c>
       <c r="C70" s="2" t="n">
-        <v>29650</v>
+        <v>29520</v>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>-$49.78K</t>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>+$145.22K</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>+$218.28K</t>
+          <t>+$205.32K</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="n">
+        <v>4451.57</v>
+      </c>
+      <c r="C71" s="2" t="n">
+        <v>406</v>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>GLD</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>-$41.04K</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>+$198.90K</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B71" s="2" t="n">
-        <v>29576.03</v>
-      </c>
-      <c r="C71" s="2" t="n">
-        <v>29520</v>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
+      <c r="B72" s="6" t="n">
+        <v>29481.03</v>
+      </c>
+      <c r="C72" s="6" t="n">
+        <v>29425</v>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>+$145.22K</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>+$205.32K</t>
-        </is>
-      </c>
-      <c r="G71" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H71" s="3" t="inlineStr">
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>+$120.18K</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>+$190.29K</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
         <is>
           <t>peak</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="n">
-        <v>4451.57</v>
-      </c>
-      <c r="C72" s="2" t="n">
-        <v>406</v>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>GLD</t>
-        </is>
-      </c>
-      <c r="E72" s="4" t="inlineStr">
-        <is>
-          <t>-$41.04K</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>+$198.90K</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
     <row r="73">
-      <c r="A73" s="7" t="inlineStr">
+      <c r="A73" s="3" t="inlineStr">
         <is>
           <t>NQ</t>
         </is>
       </c>
-      <c r="B73" s="6" t="n">
-        <v>29481.03</v>
-      </c>
-      <c r="C73" s="6" t="n">
-        <v>29425</v>
-      </c>
-      <c r="D73" s="7" t="inlineStr">
+      <c r="B73" s="2" t="n">
+        <v>29356.03</v>
+      </c>
+      <c r="C73" s="2" t="n">
+        <v>29300</v>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>+$120.18K</t>
-        </is>
-      </c>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>+$190.29K</t>
-        </is>
-      </c>
-      <c r="G73" s="7" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H73" s="7" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>-$76.59K</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>+$160.84K</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
@@ -6085,24 +6040,24 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>29356.03</v>
+        <v>29656.03</v>
       </c>
       <c r="C74" s="2" t="n">
-        <v>29300</v>
+        <v>29600</v>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E74" s="4" t="inlineStr">
-        <is>
-          <t>-$76.59K</t>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>+$66.28K</t>
         </is>
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>+$160.84K</t>
+          <t>+$154.65K</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -6119,24 +6074,24 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>29656.03</v>
+        <v>29406.03</v>
       </c>
       <c r="C75" s="2" t="n">
-        <v>29600</v>
+        <v>29350</v>
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E75" s="5" t="inlineStr">
-        <is>
-          <t>+$66.28K</t>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>-$26.51K</t>
         </is>
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>+$154.65K</t>
+          <t>+$150.23K</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -6153,24 +6108,24 @@
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>29406.03</v>
+        <v>29426.03</v>
       </c>
       <c r="C76" s="2" t="n">
-        <v>29350</v>
+        <v>29370</v>
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E76" s="4" t="inlineStr">
-        <is>
-          <t>-$26.51K</t>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>+$4.71K</t>
         </is>
       </c>
       <c r="F76" s="3" t="inlineStr">
         <is>
-          <t>+$150.23K</t>
+          <t>+$136.68K</t>
         </is>
       </c>
       <c r="G76" s="3" t="inlineStr">
@@ -6187,32 +6142,36 @@
         </is>
       </c>
       <c r="B77" s="2" t="n">
-        <v>29426.03</v>
+        <v>29636.03</v>
       </c>
       <c r="C77" s="2" t="n">
-        <v>29370</v>
+        <v>29580</v>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E77" s="5" t="inlineStr">
-        <is>
-          <t>+$4.71K</t>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>-$51.84K</t>
         </is>
       </c>
       <c r="F77" s="3" t="inlineStr">
         <is>
-          <t>+$136.68K</t>
+          <t>+$127.25K</t>
         </is>
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
@@ -6221,10 +6180,10 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>29636.03</v>
+        <v>29486.03</v>
       </c>
       <c r="C78" s="2" t="n">
-        <v>29580</v>
+        <v>29430</v>
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
@@ -6233,12 +6192,12 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
-          <t>-$51.84K</t>
+          <t>-$85.13K</t>
         </is>
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>+$127.25K</t>
+          <t>+$125.19K</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -6259,24 +6218,24 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>29486.03</v>
+        <v>29686.03</v>
       </c>
       <c r="C79" s="2" t="n">
-        <v>29430</v>
+        <v>29630</v>
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
           <t>NDX</t>
         </is>
       </c>
-      <c r="E79" s="4" t="inlineStr">
-        <is>
-          <t>-$85.13K</t>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>+$70.11K</t>
         </is>
       </c>
       <c r="F79" s="3" t="inlineStr">
         <is>
-          <t>+$125.19K</t>
+          <t>+$78.36K</t>
         </is>
       </c>
       <c r="G79" s="3" t="inlineStr">
@@ -6286,35 +6245,35 @@
       </c>
       <c r="H79" s="3" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>CL</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>29686.03</v>
+        <v>89.23</v>
       </c>
       <c r="C80" s="2" t="n">
-        <v>29630</v>
+        <v>139</v>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>NDX</t>
+          <t>USO</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>+$70.11K</t>
+          <t>+$37.59K</t>
         </is>
       </c>
       <c r="F80" s="3" t="inlineStr">
         <is>
-          <t>+$78.36K</t>
+          <t>+$43.77K</t>
         </is>
       </c>
       <c r="G80" s="3" t="inlineStr">
@@ -6324,50 +6283,12 @@
       </c>
       <c r="H80" s="3" t="inlineStr">
         <is>
-          <t>peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="3" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="n">
-        <v>89.23</v>
-      </c>
-      <c r="C81" s="2" t="n">
-        <v>139</v>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>USO</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>+$37.59K</t>
-        </is>
-      </c>
-      <c r="F81" s="3" t="inlineStr">
-        <is>
-          <t>+$43.77K</t>
-        </is>
-      </c>
-      <c r="G81" s="3" t="inlineStr">
-        <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H81" s="3" t="inlineStr">
-        <is>
           <t>valley</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H81"/>
+  <autoFilter ref="A1:H80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>